<commit_message>
updated info tab in datasets files
</commit_message>
<xml_diff>
--- a/src/microfading/datasets/2024-144_MF.BWS0025.04_G02_BW2_model_2024-08-02_MFT1.xlsx
+++ b/src/microfading/datasets/2024-144_MF.BWS0025.04_G02_BW2_model_2024-08-02_MFT1.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="info" sheetId="1" state="visible" r:id="rId2"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="139">
   <si>
     <t xml:space="preserve">parameter</t>
   </si>
@@ -36,22 +36,25 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t xml:space="preserve">author</t>
+    <t xml:space="preserve">authors</t>
   </si>
   <si>
     <t xml:space="preserve">Patin, Gauthier</t>
   </si>
   <si>
+    <t xml:space="preserve">host_institution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rijksdienst voor het Cultureel Erfgoed_Rijkserfgoed Laboratorium</t>
+  </si>
+  <si>
     <t xml:space="preserve">date_time</t>
   </si>
   <si>
-    <t xml:space="preserve">[PROJECT DATA]</t>
+    <t xml:space="preserve">comment</t>
   </si>
   <si>
-    <t xml:space="preserve">laboratorium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REL_Rijkserfgoed Laboratorium</t>
+    <t xml:space="preserve">[PROJECT INFO]</t>
   </si>
   <si>
     <t xml:space="preserve">project_id</t>
@@ -60,37 +63,49 @@
     <t xml:space="preserve">2024-144</t>
   </si>
   <si>
-    <t xml:space="preserve">projectleider</t>
+    <t xml:space="preserve">institution</t>
   </si>
   <si>
-    <t xml:space="preserve">meelezer</t>
+    <t xml:space="preserve">Rijksmuseum Amsterdam</t>
   </si>
   <si>
-    <t xml:space="preserve">Brokerhof, Agnes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aanvraagdatum</t>
+    <t xml:space="preserve">start_date</t>
   </si>
   <si>
     <t xml:space="preserve">2024-06-03</t>
   </si>
   <si>
-    <t xml:space="preserve">uiterste_datum</t>
+    <t xml:space="preserve">end_date</t>
   </si>
   <si>
     <t xml:space="preserve">2024-10-30</t>
   </si>
   <si>
-    <t xml:space="preserve">comment</t>
+    <t xml:space="preserve">project_leader</t>
   </si>
   <si>
-    <t xml:space="preserve">[OBJECT DATA]</t>
+    <t xml:space="preserve">GP</t>
   </si>
   <si>
-    <t xml:space="preserve">institution</t>
+    <t xml:space="preserve">co-researchers</t>
   </si>
   <si>
-    <t xml:space="preserve">RMA_Rijksmuseum Amsterdam</t>
+    <t xml:space="preserve">AB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">keywords</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Japans-prenten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">methods</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MFT_Photo_RIS_RS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[OBJECT INFO]</t>
   </si>
   <si>
     <t xml:space="preserve">object_id</t>
@@ -141,7 +156,31 @@
     <t xml:space="preserve">2023</t>
   </si>
   <si>
-    <t xml:space="preserve">object_support</t>
+    <t xml:space="preserve">object_owner</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">R</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ijkserfgoed Laboratorium</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">object_material</t>
   </si>
   <si>
     <t xml:space="preserve">wool</t>
@@ -177,7 +216,7 @@
     <t xml:space="preserve">status</t>
   </si>
   <si>
-    <t xml:space="preserve">[DEVICE DATA]</t>
+    <t xml:space="preserve">[DEVICE INFO]</t>
   </si>
   <si>
     <t xml:space="preserve">device</t>
@@ -258,7 +297,7 @@
     <t xml:space="preserve">WR1_Dr Lange LZM 013, pressed barium sulphate powder</t>
   </si>
   <si>
-    <t xml:space="preserve">[ANALYSIS DATA]</t>
+    <t xml:space="preserve">[ANALYSIS INFO]</t>
   </si>
   <si>
     <t xml:space="preserve">meas_id</t>
@@ -267,34 +306,19 @@
     <t xml:space="preserve">MF.BWS0025.04</t>
   </si>
   <si>
-    <t xml:space="preserve">group</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">group_description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">background</t>
-  </si>
-  <si>
     <t xml:space="preserve">specular_component</t>
   </si>
   <si>
     <t xml:space="preserve">partially included</t>
   </si>
   <si>
-    <t xml:space="preserve">integration_time_ms</t>
+    <t xml:space="preserve">integration_time_sample_ms</t>
   </si>
   <si>
-    <t xml:space="preserve">124.00</t>
+    <t xml:space="preserve">integration_time_whitestandard_ms</t>
   </si>
   <si>
     <t xml:space="preserve">average</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20</t>
   </si>
   <si>
     <t xml:space="preserve">duration_min</t>
@@ -304,9 +328,6 @@
   </si>
   <si>
     <t xml:space="preserve">measurements_N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">61</t>
   </si>
   <si>
     <t xml:space="preserve">illuminant</t>
@@ -321,7 +342,37 @@
     <t xml:space="preserve">10deg</t>
   </si>
   <si>
-    <t xml:space="preserve">[BEAM DATA]</t>
+    <t xml:space="preserve">[SPOT INFO]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spot_group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spot_description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spot_color</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spot_components</t>
+  </si>
+  <si>
+    <t xml:space="preserve">background</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bbg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spot_image</t>
+  </si>
+  <si>
+    <t xml:space="preserve">other_analyses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[BEAM INFO]</t>
   </si>
   <si>
     <t xml:space="preserve">beam_photo</t>
@@ -342,67 +393,31 @@
     <t xml:space="preserve">unknown</t>
   </si>
   <si>
-    <t xml:space="preserve">power_mW</t>
+    <t xml:space="preserve">radiantFlux_mW</t>
   </si>
   <si>
     <t xml:space="preserve">P.00037_5.726+/-0.006</t>
   </si>
   <si>
-    <t xml:space="preserve">irradiance_W/m**2</t>
+    <t xml:space="preserve">irradiance_He_W/m^2</t>
   </si>
   <si>
     <t xml:space="preserve">(2.9+/-0.5)e+03</t>
   </si>
   <si>
-    <t xml:space="preserve">luminuous_flux_lm</t>
+    <t xml:space="preserve">luminuousFlux_lm</t>
   </si>
   <si>
-    <t xml:space="preserve">illuminance_Mlx</t>
+    <t xml:space="preserve">illuminance_Hv_Mlx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">radiantExposure_He_MJ/m^2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exposureDose_Hv_Mlxh</t>
   </si>
   <si>
     <t xml:space="preserve">[RESULTS]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">totalDose_He_MJ/m**2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">totalDose_Hv_Mlxh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fittedEqHe_dE00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">y = 0.373*(x**0.294)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fittedEqHv_dE00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">y = 0.731*(x**0.294)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fittedRate_dE00_at_2Mlxh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fittedRate_dE00_at_20MJ/m**2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dE00_at_300klxh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dE00_at_3MJ/m**2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dEab_final</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dE00_final</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dR_VIS_final</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hv_at_1dE00</t>
   </si>
   <si>
     <t xml:space="preserve">BWSE</t>
@@ -452,7 +467,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -481,6 +496,18 @@
       <name val="Cambria"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Cambria"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -532,7 +559,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -546,6 +573,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -566,8 +601,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B82"/>
-  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:B1048576"/>
+  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="48.07"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -593,399 +631,403 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="3" t="n">
-        <v>45506.6439583333</v>
+      <c r="B4" s="0" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>3</v>
+        <v>8</v>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>45506.6439583333</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="B6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="B8" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="B12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B13" s="5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B14" s="5" t="s">
         <v>24</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>26</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>49</v>
+        <v>52</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>3</v>
+        <v>55</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>57</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B35" s="2" t="n">
-        <v>1</v>
+        <v>59</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B37" s="2" t="n">
-        <v>24</v>
+        <v>63</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B38" s="2" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>3</v>
+        <v>81</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>34</v>
+        <v>3</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>90</v>
+      </c>
+      <c r="B53" s="2" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
+      </c>
+      <c r="B54" s="2" t="n">
+        <v>124</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>20</v>
@@ -993,7 +1035,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>20</v>
@@ -1001,103 +1043,95 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="B57" s="2" t="s">
         <v>94</v>
+      </c>
+      <c r="B57" s="2" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B58" s="2" t="s">
-        <v>96</v>
+      <c r="B58" s="2" t="n">
+        <v>61</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B59" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B60" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B60" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B61" s="2" t="s">
+      <c r="B61" s="2"/>
+    </row>
+    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="2" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="2" t="s">
+      <c r="B62" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B62" s="2" t="n">
-        <v>0.5404</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B63" s="2" t="n">
-        <v>1423</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B63" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
         <v>104</v>
       </c>
       <c r="B64" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="2" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="2" t="s">
+      <c r="B65" s="2"/>
+    </row>
+    <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="B65" s="2" t="s">
+      <c r="B66" s="2" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="2" t="s">
+    <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B66" s="2" t="s">
+      <c r="B67" s="2"/>
+    </row>
+    <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="2" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="B67" s="2" t="n">
-        <v>1.68</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="B68" s="2" t="n">
-        <v>1.0583</v>
-      </c>
+      <c r="B68" s="2"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>3</v>
@@ -1105,50 +1139,50 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B70" s="2" t="n">
-        <v>3.4</v>
+        <v>111</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B71" s="2" t="n">
-        <v>0.34465</v>
+        <v>0.5404</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="B72" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
+      </c>
+      <c r="B72" s="2" t="n">
+        <v>1423</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="B74" s="2" t="n">
-        <v>0.134</v>
+        <v>117</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B75" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="B75" s="2" t="n">
-        <v>0.013</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1156,7 +1190,7 @@
         <v>121</v>
       </c>
       <c r="B76" s="2" t="n">
-        <v>0.516</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1164,31 +1198,31 @@
         <v>122</v>
       </c>
       <c r="B77" s="2" t="n">
-        <v>0.518</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1.0583</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
         <v>123</v>
       </c>
       <c r="B78" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
         <v>124</v>
       </c>
       <c r="B79" s="2" t="n">
-        <v>0.55</v>
+        <v>0.34465</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B80" s="2" t="n">
-        <v>0.609</v>
+      <c r="B80" s="2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1196,17 +1230,13 @@
         <v>126</v>
       </c>
       <c r="B81" s="2" t="n">
-        <v>28.565</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="B82" s="2" t="n">
         <v>4.91</v>
       </c>
     </row>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1224,41 +1254,41 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K37"/>
-  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2538,11 +2568,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AJ792"/>
-  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B1" s="1" t="n">
         <v>0</v>

</xml_diff>